<commit_message>
FSI vulnerability heat map and FSAP reports for GCC countries
- FSI: add deposits to loans, liquid assets to total assets, FX loans and
  liabilities, large exposures, commercial real estate loans, household
  debt; each indicator has a group and a vulnerability direction
- Heat map: grouped rows, no 'higher = safer' labels, vulnerability
  wording, layout fixed
- FSAP: catalog of 21 IMF FSAP reports for GCC countries (fsap_reports.csv,
  IMF_FSAP_reports_catalog.xlsx) and agent instructions to answer from
  the report PDFs with citations

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/m365-agent/Agent_tools.xlsx
+++ b/m365-agent/Agent_tools.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A165"/>
+  <dimension ref="A1:A175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1193,306 +1193,376 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>FSI_ORDER = ['FSI688_CFSI_PT', 'FSI626_CFSI_PT', 'FSI15_CFSI_PT', 'T1KTA_CFSI_PT', 'AQ12_CFSI_PT', 'FSI17_CFSI_PT',</t>
+          <t># Groups and directions come from the FSI workbook: column Group, and column "More vulnerable when"</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">             'AQ14_CFSI_PT', 'AQ1_CFSI_PT', 'FSI524_CFSI_PT', 'ROA_CFSI_PT', 'ROE_CFSI_PT', 'FSI99_CFSI_PT',</t>
+          <t># ("higher" or "lower"), set from a financial-sector vulnerability perspective.</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t xml:space="preserve">             'FSI107_CFSI_PT', 'FSI765_CFSI_PT', 'FSI288_CFSI_PT', 'FSI289_CFSI_PT', 'FSI555_CFSI_PT']</t>
-        </is>
-      </c>
+      <c r="A122" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t># Higher value = MORE risk for these; for all others a higher value = LESS risk (rank is flipped).</t>
-        </is>
-      </c>
+      <c r="A123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>RISK_UP = {'AQ12_CFSI_PT', 'FSI17_CFSI_PT', 'AQ1_CFSI_PT', 'FSI524_CFSI_PT', 'FSI107_CFSI_PT', 'FSI555_CFSI_PT'}</t>
+          <t>def percent_rank(s):</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
+      <c r="A125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    """Excel PERCENTRANK.INC of every value within its own series: (values below) / (n - 1)."""</t>
+        </is>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr"/>
+      <c r="A126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    s = s.dropna(); return (s.rank(method='min') - 1) / (len(s) - 1) if len(s) &gt; 1 else s * np.nan</t>
+        </is>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>def percent_rank(s):</t>
-        </is>
-      </c>
+      <c r="A127" t="inlineStr"/>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    """Excel PERCENTRANK.INC of every value within its own series: (values below) / (n - 1)."""</t>
-        </is>
-      </c>
+      <c r="A128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">    s = s.dropna(); return (s.rank(method='min') - 1) / (len(s) - 1) if len(s) &gt; 1 else s * np.nan</t>
+          <t>def fsi_heatmap(country, quarters=12, min_history=8):</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr"/>
+      <c r="A130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    """Heat map of FSIs: colour = vulnerability percentile vs the country's own history</t>
+        </is>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr"/>
+      <c r="A131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    (0 = least vulnerable ever, dark blue; 1 = most vulnerable ever, dark red); cells show actual values."""</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>def fsi_heatmap(country, quarters=12, min_history=8):</t>
+          <t xml:space="preserve">    rows = F[(F['Economy'].str.lower() == country.lower()) | (F['Economy code'] == country.upper())]</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Heat map of core FSIs: colour = risk percentile vs the country's own history</t>
+          <t xml:space="preserve">    rows = rows.drop_duplicates('Indicator code').set_index('Indicator code')</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (0 = lowest risk ever, dark blue; 1 = highest risk ever, dark red); cells show actual values."""</t>
+          <t xml:space="preserve">    per = [c for c in rows.columns if re.fullmatch(r'\d{4}-Q\d', str(c))]</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">    rows = F[(F['Economy'].str.lower() == country.lower()) | (F['Economy code'] == country.upper())]</t>
+          <t xml:space="preserve">    V = rows[per].apply(pd.to_numeric, errors='coerce')</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">    rows = rows.set_index('Indicator code').reindex([c for c in FSI_ORDER if c in set(rows['Indicator code'])])</t>
+          <t xml:space="preserve">    V = V[V.notna().sum(axis=1) &gt;= min_history]</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">    per = [c for c in rows.columns if re.fullmatch(r'\d{4}-Q\d', str(c))]</t>
+          <t xml:space="preserve">    rows = rows.loc[V.index]</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">    V = rows[per].apply(pd.to_numeric, errors='coerce')</t>
+          <t xml:space="preserve">    R = V.apply(percent_rank, axis=1).reindex(columns=per)</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">    V = V[V.notna().sum(axis=1) &gt;= min_history]</t>
+          <t xml:space="preserve">    lower = (rows['More vulnerable when'] == 'lower').values; R.loc[lower] = 1 - R.loc[lower]</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">    R = V.apply(percent_rank, axis=1).reindex(columns=per)</t>
+          <t xml:space="preserve">    first = min(V.apply(lambda r: r.first_valid_index(), axis=1).dropna())</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">    safer = ~R.index.isin(list(RISK_UP)); R.loc[safer] = 1 - R.loc[safer]</t>
+          <t xml:space="preserve">    cols = [c for c in per if V[c].notna().any()][-quarters:]</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">    first = min(V.apply(lambda r: r.first_valid_index(), axis=1).dropna())</t>
+          <t xml:space="preserve">    V, R = V[cols], R[cols]</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cols = [c for c in per if V[c].notna().any()][-quarters:]</t>
+          <t xml:space="preserve">    # explicit layout in inches: labels left, group names right, colour bar and source below</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">    V, R = V[cols], R[cols]</t>
+          <t xml:space="preserve">    L = 0.3 + 0.062 * rows['Indicator'].str.len().max(); Rt = 0.4 + 0.07 * rows['Group'].str.len().max()</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">    fig, ax = plt.subplots(figsize=(4.5 + 0.7 * len(cols), 1.4 + 0.42 * len(V)))</t>
+          <t xml:space="preserve">    w, h, top, bot = 0.7 * len(cols), 0.42 * len(V), 0.75, 1.75</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">    im = ax.imshow(R.values.astype(float), cmap='RdBu_r', vmin=0, vmax=1, aspect='auto')</t>
+          <t xml:space="preserve">    W, H = L + w + Rt, top + h + bot</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">    for i in range(len(V)):</t>
+          <t xml:space="preserve">    fig = plt.figure(figsize=(W, H)); ax = fig.add_axes([L / W, bot / H, w / W, h / H])</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for j in range(len(cols)):</t>
+          <t xml:space="preserve">    im = ax.imshow(R.values.astype(float), cmap='RdBu_r', vmin=0, vmax=1, aspect='auto')</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">            v, r = V.iat[i, j], R.iat[i, j]</t>
+          <t xml:space="preserve">    for i in range(len(V)):</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if pd.notna(v):</t>
+          <t xml:space="preserve">        for j in range(len(cols)):</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">                ax.text(j, i, f'{v:.1f}', ha='center', va='center', fontsize=8,</t>
+          <t xml:space="preserve">            v, r = V.iat[i, j], R.iat[i, j]</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">                        color='white' if pd.notna(r) and abs(r - 0.5) &gt; 0.3 else 'black')</t>
+          <t xml:space="preserve">            if pd.notna(v):</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">    labels = [f"{rows.at[c, 'Indicator']} ({'higher = riskier' if c in RISK_UP else 'higher = safer'})" for c in V.index]</t>
+          <t xml:space="preserve">                ax.text(j, i, f'{v:.1f}', ha='center', va='center', fontsize=8,</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax.set_yticks(range(len(V))); ax.set_yticklabels(labels, fontsize=8)</t>
+          <t xml:space="preserve">                        color='white' if pd.notna(r) and abs(r - 0.5) &gt; 0.3 else 'black')</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax.set_xticks(range(len(cols))); ax.set_xticklabels(cols, rotation=45, ha='right', fontsize=8)</t>
+          <t xml:space="preserve">    ax.set_yticks(range(len(V))); ax.set_yticklabels(rows['Indicator'], fontsize=8)</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cb = fig.colorbar(im, ax=ax, fraction=0.03, pad=0.02); cb.set_ticks([0, 0.5, 1])</t>
+          <t xml:space="preserve">    ax.set_xticks(range(len(cols))); ax.set_xticklabels(cols, rotation=45, ha='right', fontsize=8)</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cb.set_ticklabels(['Lower risk', 'Median', 'Higher risk'])</t>
+          <t xml:space="preserve">    groups = list(rows['Group'])</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax.set_title(f"{rows['Economy'].dropna().iloc[0]}: financial soundness heat map\n"</t>
+          <t xml:space="preserve">    starts = [i for i in range(len(groups)) if i == 0 or groups[i] != groups[i - 1]]</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 "colour = percent rank vs own history (dark red = highest risk, dark blue = lowest)",</t>
+          <t xml:space="preserve">    for i in starts[1:]: ax.axhline(i - 0.5, color='black', lw=1.2)</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 loc='left', weight='bold', color=BLUE, fontsize=10)</t>
+          <t xml:space="preserve">    ax2 = ax.twinx(); ax2.set_ylim(ax.get_ylim())</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">    note =f"Each indicator is ranked against all its own quarters since {first} (Excel PERCENTRANK.INC)."</t>
+          <t xml:space="preserve">    ax2.set_yticks([(s + e - 1) / 2 for s, e in zip(starts, starts[1:] + [len(groups)])])</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">    _footer(fig, f"Source: {rows['Citation'].dropna().iloc[0]}. {note}")</t>
+          <t xml:space="preserve">    ax2.set_yticklabels([groups[s] for s in starts], fontsize=8, weight='bold', color=BLUE)</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">    return pd.DataFrame({'Latest value': V.ffill(axis=1).iloc[:, -1],</t>
+          <t xml:space="preserve">    ax2.tick_params(length=0); ax2.spines[:].set_visible(False)</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">                         'Risk percentile': R.ffill(axis=1).iloc[:, -1].round(2)},).set_index(pd.Index(</t>
+          <t xml:space="preserve">    cax = fig.add_axes([L / W, 0.55 / H, min(w, 5) / W, 0.13 / H])</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">                         [rows.at[c, 'Indicator'] for c in V.index], name='Indicator'))</t>
+          <t xml:space="preserve">    cb = fig.colorbar(im, cax=cax, orientation='horizontal'); cb.set_ticks([0, 0.5, 1])</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    cb.set_ticklabels(['Less vulnerable', 'Median', 'More vulnerable']); cb.ax.tick_params(labelsize=8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ax.set_title(f"{rows['Economy'].dropna().iloc[0]}: financial soundness heat map\n"</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 "colour = percent rank vs own history (dark red = most vulnerable, dark blue = least)",</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 loc='left', weight='bold', color=BLUE, fontsize=10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    note = f"Each indicator is ranked against all its own quarters since {first} (Excel PERCENTRANK.INC)."</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    fig.text(0.01, 0.06 / H, textwrap.fill(f"Source: {rows['Citation'].dropna().iloc[0]}. {note}", int(W * 14)),</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             fontsize=8, color='dimgray'); plt.show()</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    return pd.DataFrame({'Group': rows['Group'].values, 'Indicator': rows['Indicator'].values,</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         'Latest value': V.ffill(axis=1).iloc[:, -1].round(2).values,</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         'Vulnerability percentile': R.ffill(axis=1).iloc[:, -1].round(2).values})</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M365 agent: code in every workbook, no-Python fallback, quoted FSAP evidence
- The agent code is now also in a 'Code' sheet of every workbook and loads
  whichever workbooks are available (Copilot may pass only some files to
  Code interpreter); step 1 finds the code in any workbook
- Summary sheets readable without Python: WEO GCC_Summary, FSI Latest
  (vulnerability percentiles), credit Latest (ratio, trend, gap)
- Instructions: fallback when Code interpreter is unavailable; FSAP answers
  quote the supporting paragraph with the key sentence in bold, plus
  title, page and link

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/m365-agent/Agent_tools.xlsx
+++ b/m365-agent/Agent_tools.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A175"/>
+  <dimension ref="A1:A189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,565 +434,557 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t># build_data_file.py stores this file, one line per row, in Agent_tools.xlsx (sheet "Code");</t>
+          <t># build_data_file.py stores this file, one line per row, in a sheet "Code" of every workbook</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t># the agent runs it with exec(). Keep it self-contained (pandas, numpy, matplotlib only).</t>
+          <t># (and in Agent_tools.xlsx); the agent runs it with exec(). Keep it self-contained</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>import glob, re, textwrap, numpy as np, pandas as pd, matplotlib.pyplot as plt</t>
+          <t># (pandas, numpy, matplotlib only).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>import glob, os, re, textwrap, numpy as np, pandas as pd, matplotlib.pyplot as plt</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>from matplotlib.ticker import MaxNLocator</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-    </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>fs = glob.glob('/mnt/data/*.xlsx') + glob.glob('**/*.xlsx', recursive=True)</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>xl = lambda k, sh: pd.read_excel(next(p for p in fs if k in p), sheet_name=sh)</t>
+          <t>fs = sorted({os.path.abspath(p) for pat in ('/mnt/**/*.xls*', '/home/**/*.xls*', '**/*.xls*')</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>D, G = xl('World_Economic_Outlook', 'Data'), xl('World_Economic_Outlook', 'Groups')</t>
+          <t xml:space="preserve">             for p in glob.glob(pat, recursive=True)})</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>F = xl('Financial_Soundness', 'FSI_Quarterly')</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CQ, CA = xl('BIS_credit', 'Credit_GDP_Quarterly'), xl('BIS_credit', 'Credit_GDP_Annual')</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>M = xl('IMF_MFS_credit', 'Credit_GDP_Annual')</t>
+          <t>def xl(key, sheet):</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BLUE, RED = '#4B82AD', '#c0392b'</t>
+          <t xml:space="preserve">    """Load a sheet from the first workbook whose name contains `key`; None if not available."""</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PERIOD = re.compile(r'\d{4}(-Q\d)?')</t>
+          <t xml:space="preserve">    p = next((p for p in fs if key in os.path.basename(p)), None)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    return pd.read_excel(p, sheet_name=sheet) if p else None</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>def _style(ax):</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax.grid(alpha=0.3); ax.spines[['top', 'right']].set_visible(False)</t>
+          <t>D, G = xl('World_Economic_Outlook', 'Data'), xl('World_Economic_Outlook', 'Groups')</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>F = xl('Financial_Soundness', 'FSI_Quarterly')</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CQ, CA = xl('BIS_credit', 'Credit_GDP_Quarterly'), xl('BIS_credit', 'Credit_GDP_Annual')</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>def _footer(fig, src):</t>
+          <t>M = xl('IMF_MFS_credit', 'Credit_GDP_Annual')</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    fig.text(0.01, 0.01, textwrap.fill(src, 150), fontsize=8, color='dimgray')</t>
+          <t>_loaded = {'D (IMF WEO)': D, 'G (groups)': G, 'F (FSI)': F, 'CQ/CA (BIS credit)': CQ, 'M (Gulf MFS credit)': M}</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    fig.tight_layout(rect=(0, 0.06, 1, 1)); plt.show()</t>
+          <t>print('Loaded:', ', '.join(k for k, v in _loaded.items() if v is not None) or 'no data workbooks')</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>if any(v is None for v in _loaded.values()):</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    print('Not available:', ', '.join(k for k, v in _loaded.items() if v is None),</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t># --------------------------------------------------------------------------- charts</t>
+          <t xml:space="preserve">          '| workbooks found:', [os.path.basename(p) for p in fs])</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>def chart(rows, start=2000, end=2031, kind='line', year=None):</t>
+          <t>BLUE, RED = '#4B82AD', '#c0392b'</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """kind='line' time series; 'bar' ranking for one period; 'gap' credit-to-GDP ratio + HP trend</t>
+          <t>PERIOD = re.compile(r'\d{4}(-Q\d)?')</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    (top) and gap (bottom) - pass the 3 rows CREDIT_GDP, CREDIT_GDP_TREND, CREDIT_GDP_GAP."""</t>
-        </is>
-      </c>
+      <c r="A30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    r0 = rows.iloc[-1]; P = int(r0['First projection year']) if 'First projection year' in rows else None</t>
-        </is>
-      </c>
+      <c r="A31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">    per = [c for c in rows.columns if PERIOD.fullmatch(str(c)) and start &lt;= int(str(c)[:4]) &lt;= end]</t>
+          <t>def _style(ax):</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    x = [int(c[:4]) + (int(c[-1]) - 1) / 4 if '-Q' in c else int(c) for c in per]</t>
+          <t xml:space="preserve">    ax.grid(alpha=0.3); ax.spines[['top', 'right']].set_visible(False)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    V = rows[per].apply(pd.to_numeric, errors='coerce'); codes = list(rows['Indicator code'])</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    many = rows['Indicator'].nunique() &gt; 1; title = r0['Economy'] if many else r0['Indicator']</t>
-        </is>
-      </c>
+      <c r="A35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">    L = str(r0.get('Source link') or ''); src = f"Source: {r0['Citation']}. {L.rsplit('/', 1)[0] if '@' in L else L}"</t>
+          <t>def _footer(fig, src):</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if kind == 'gap':</t>
+          <t xml:space="preserve">    fig.text(0.01, 0.01, textwrap.fill(src, 150), fontsize=8, color='dimgray')</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">        fig, (ax, a2) = plt.subplots(2, 1, figsize=(10, 7.5), sharex=True, gridspec_kw={'height_ratios': [2, 1]})</t>
+          <t xml:space="preserve">    fig.tight_layout(rect=(0, 0.06, 1, 1)); plt.show()</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        for c, lab, ls in (('CREDIT_GDP', 'Credit-to-GDP ratio', '-'), ('CREDIT_GDP_TREND', 'Hodrick-Prescott trend', '--')):</t>
-        </is>
-      </c>
+      <c r="A39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            ax.plot(x, V.values[codes.index(c)], lw=2, ls=ls, label=lab)</t>
-        </is>
-      </c>
+      <c r="A40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">        g = V.values[codes.index('CREDIT_GDP_GAP')]</t>
+          <t># --------------------------------------------------------------------------- charts</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">        a2.bar(x, g, width=0.22 if '-Q' in per[0] else 0.8, color=[RED if v &gt;= 0 else BLUE for v in g])</t>
+          <t>def chart(rows, start=2000, end=2031, kind='line', year=None):</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for h in (2, 10): a2.axhline(h, color='grey', ls=':', lw=1)</t>
+          <t xml:space="preserve">    """kind='line' time series; 'bar' ranking for one period; 'gap' credit-to-GDP ratio + HP trend</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">        a2.axhline(0, color='black', lw=0.8); a2.set_ylabel('Gap, pp of GDP')</t>
+          <t xml:space="preserve">    (top) and gap (bottom) - pass the 3 rows CREDIT_GDP, CREDIT_GDP_TREND, CREDIT_GDP_GAP."""</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">        _style(a2); a2.xaxis.set_major_locator(MaxNLocator(integer=True))</t>
+          <t xml:space="preserve">    r0 = rows.iloc[-1]; P = int(r0['First projection year']) if 'First projection year' in rows else None</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ax.set_ylabel('Percent of GDP'); ax.legend(frameon=False)</t>
+          <t xml:space="preserve">    per = [c for c in rows.columns if PERIOD.fullmatch(str(c)) and start &lt;= int(str(c)[:4]) &lt;= end]</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">        title = f"{r0['Economy']}: credit-to-GDP ratio, trend and gap"</t>
+          <t xml:space="preserve">    x = [int(c[:4]) + (int(c[-1]) - 1) / 4 if '-Q' in c else int(c) for c in per]</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">    else:</t>
+          <t xml:space="preserve">    V = rows[per].apply(pd.to_numeric, errors='coerce'); codes = list(rows['Indicator code'])</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">        fig, ax = plt.subplots(figsize=(10, 5.5))</t>
+          <t xml:space="preserve">    many = rows['Indicator'].nunique() &gt; 1; title = r0['Economy'] if many else r0['Indicator']</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if kind == 'bar':</t>
+          <t xml:space="preserve">    L = str(r0.get('Source link') or ''); src = f"Source: {r0['Citation']}. {L.rsplit('/', 1)[0] if '@' in L else L}"</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">        n = V.notna().sum(); y = str(year) if year else (str(P - 1) if P else n[n &gt;= 0.8 * n.max()].index[-1])</t>
+          <t xml:space="preserve">    if kind == 'gap':</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">        s = rows.set_index('Economy')[y].dropna().sort_values()</t>
+          <t xml:space="preserve">        fig, (ax, a2) = plt.subplots(2, 1, figsize=(10, 7.5), sharex=True, gridspec_kw={'height_ratios': [2, 1]})</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ax.barh(s.index, s.values, color='#2a6fb0'); ax.set_xlabel(r0['Unit'])</t>
+          <t xml:space="preserve">        for c, lab, ls in (('CREDIT_GDP', 'Credit-to-GDP ratio', '-'), ('CREDIT_GDP_TREND', 'Hodrick-Prescott trend', '--')):</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">        title = f"{title}, {y}" + (' (IMF projection)' if P and int(y[:4]) &gt;= P else '')</t>
+          <t xml:space="preserve">            ax.plot(x, V.values[codes.index(c)], lw=2, ls=ls, label=lab)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    elif kind == 'line':</t>
+          <t xml:space="preserve">        g = V.values[codes.index('CREDIT_GDP_GAP')]</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for lab, v in zip(rows['Indicator'] if many else rows['Economy'], V.values):</t>
+          <t xml:space="preserve">        a2.bar(x, g, width=0.22 if '-Q' in per[0] else 0.8, color=[RED if v &gt;= 0 else BLUE for v in g])</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">            ax.plot(x, v, lw=2, label=lab)</t>
+          <t xml:space="preserve">        for h in (2, 10): a2.axhline(h, color='grey', ls=':', lw=1)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if V.min().min() &lt; 0 &lt; V.max().max(): ax.axhline(0, color='black', lw=0.8)</t>
+          <t xml:space="preserve">        a2.axhline(0, color='black', lw=0.8); a2.set_ylabel('Gap, pp of GDP')</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if P and x[-1] &gt;= P:</t>
+          <t xml:space="preserve">        _style(a2); a2.xaxis.set_major_locator(MaxNLocator(integer=True))</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">            ax.axvspan(P - 0.5, x[-1] + 0.5, color='grey', alpha=0.15, zorder=0)</t>
+          <t xml:space="preserve">        ax.set_ylabel('Percent of GDP'); ax.legend(frameon=False)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">            ax.text(P, 0.98, ' IMF projections', transform=ax.get_xaxis_transform(), va='top', fontsize=9, color='dimgray')</t>
+          <t xml:space="preserve">        title = f"{r0['Economy']}: credit-to-GDP ratio, trend and gap"</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ax.set_ylabel(r0['Unit']); ax.legend(frameon=False); ax.xaxis.set_major_locator(MaxNLocator(integer=True))</t>
+          <t xml:space="preserve">    else:</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax.set_title(title, loc='left', weight='bold', color=BLUE); _style(ax)</t>
+          <t xml:space="preserve">        fig, ax = plt.subplots(figsize=(10, 5.5))</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">    _footer(fig, src)</t>
+          <t xml:space="preserve">    if kind == 'bar':</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr"/>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        n = V.notna().sum(); y = str(year) if year else (str(P - 1) if P else n[n &gt;= 0.8 * n.max()].index[-1])</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        s = rows.set_index('Economy')[y].dropna().sort_values()</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t># --------------------------------------------------------------------------- user data: credit gap</t>
+          <t xml:space="preserve">        ax.barh(s.index, s.values, color='#2a6fb0'); ax.set_xlabel(r0['Unit'])</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>def hp_one_sided(y, lamb):</t>
+          <t xml:space="preserve">        title = f"{title}, {y}" + (' (IMF projection)' if P and int(y[:4]) &gt;= P else '')</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """One-sided HP trend: for each t, fit a standard HP filter on y[0..t] and keep the last value."""</t>
+          <t xml:space="preserve">    elif kind == 'line':</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">    y = np.asarray(y, float); out = np.full(len(y), np.nan)</t>
+          <t xml:space="preserve">        for lab, v in zip(rows['Indicator'] if many else rows['Economy'], V.values):</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">    for t in range(1, len(y) + 1):</t>
+          <t xml:space="preserve">            ax.plot(x, v, lw=2, label=lab)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if t &lt; 3:</t>
+          <t xml:space="preserve">        if V.min().min() &lt; 0 &lt; V.max().max(): ax.axhline(0, color='black', lw=0.8)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">            out[t - 1] = y[t - 1]; continue</t>
+          <t xml:space="preserve">        if P and x[-1] &gt;= P:</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">        d = np.diff(np.eye(t), 2, axis=0)</t>
+          <t xml:space="preserve">            ax.axvspan(P - 0.5, x[-1] + 0.5, color='grey', alpha=0.15, zorder=0)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">        out[t - 1] = np.linalg.solve(np.eye(t) + lamb * d.T @ d, y[:t])[-1]</t>
+          <t xml:space="preserve">            ax.text(P, 0.98, ' IMF projections', transform=ax.get_xaxis_transform(), va='top', fontsize=9, color='dimgray')</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">    return out</t>
+          <t xml:space="preserve">        ax.set_ylabel(r0['Unit']); ax.legend(frameon=False); ax.xaxis.set_major_locator(MaxNLocator(integer=True))</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ax.set_title(title, loc='left', weight='bold', color=BLUE); _style(ax)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    _footer(fig, src)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>def to_periods(index):</t>
-        </is>
-      </c>
+      <c r="A79" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    """Dates / 2020 / '2020Q1' / '2020-Q1' -&gt; '2020' or '2020-Q1'. Dates become quarters; a series</t>
-        </is>
-      </c>
+      <c r="A80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">    with only one date per year (e.g. every 31 Dec) becomes annual."""</t>
+          <t># --------------------------------------------------------------------------- user data: credit gap</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">    out = []</t>
+          <t>def hp_one_sided(y, lamb):</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">    for v in index:</t>
+          <t xml:space="preserve">    """One-sided HP trend: for each t, fit a standard HP filter on y[0..t] and keep the last value."""</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">        s = str(v).strip().upper().replace(' ', '')</t>
+          <t xml:space="preserve">    y = np.asarray(y, float); out = np.full(len(y), np.nan)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if re.fullmatch(r'\d{4}(\.0)?', s): out.append(s[:4])</t>
+          <t xml:space="preserve">    for t in range(1, len(y) + 1):</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">        elif re.fullmatch(r'\d{4}-?Q[1-4]', s): out.append(f'{s[:4]}-Q{s[-1]}')</t>
+          <t xml:space="preserve">        if t &lt; 3:</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">        else: t = pd.Timestamp(v); out.append(f'{t.year}-Q{t.quarter}')</t>
+          <t xml:space="preserve">            out[t - 1] = y[t - 1]; continue</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if all('-Q' in p for p in out) and len({p[:4] for p in out}) == len(out):</t>
+          <t xml:space="preserve">        d = np.diff(np.eye(t), 2, axis=0)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">        out = [p[:4] for p in out]</t>
+          <t xml:space="preserve">        out[t - 1] = np.linalg.solve(np.eye(t) + lamb * d.T @ d, y[:t])[-1]</t>
         </is>
       </c>
     </row>
@@ -1012,555 +1004,645 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>def user_gap(credit=None, gdp=None, ratio=None, economy='User data', lamb=None, min_years=10, source='User-provided data'):</t>
+          <t>def to_periods(index):</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Build the 3 gap rows from the user's own data, ready for chart(rows, kind='gap').</t>
+          <t xml:space="preserve">    """Dates / 2020 / '2020Q1' / '2020-Q1' -&gt; '2020' or '2020-Q1'. Dates become quarters; a series</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Give either `ratio` (% of GDP) or `credit` and `gdp` as pandas Series indexed by period/date.</t>
+          <t xml:space="preserve">    with only one date per year (e.g. every 31 Dec) becomes annual."""</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Quarterly GDP is summed over the last 4 quarters (BIS method); annual GDP with quarterly credit</t>
+          <t xml:space="preserve">    out = []</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">    is matched by calendar year. lambda: 400,000 quarterly, 100,000 annual (override with lamb)."""</t>
+          <t xml:space="preserve">    for v in index:</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if ratio is None:</t>
+          <t xml:space="preserve">        s = str(v).strip().upper().replace(' ', '')</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">        c = pd.Series(credit.values, index=to_periods(credit.index), dtype=float).dropna()</t>
+          <t xml:space="preserve">        if re.fullmatch(r'\d{4}(\.0)?', s): out.append(s[:4])</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">        g = pd.Series(gdp.values, index=to_periods(gdp.index), dtype=float).dropna()</t>
+          <t xml:space="preserve">        elif re.fullmatch(r'\d{4}-?Q[1-4]', s): out.append(f'{s[:4]}-Q{s[-1]}')</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">        qc, qg = '-Q' in c.index[0], '-Q' in g.index[0]</t>
+          <t xml:space="preserve">        else: t = pd.Timestamp(v); out.append(f'{t.year}-Q{t.quarter}')</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if qc and qg: g = g.sort_index().rolling(4).sum()</t>
+          <t xml:space="preserve">    if all('-Q' in p for p in out) and len({p[:4] for p in out}) == len(out):</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">        elif qc: g = pd.Series(g.reindex([p[:4] for p in c.index]).values, index=c.index)</t>
+          <t xml:space="preserve">        out = [p[:4] for p in out]</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ratio = 100 * c / g.reindex(c.index)</t>
+          <t xml:space="preserve">    return out</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    else:</t>
-        </is>
-      </c>
+      <c r="A105" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ratio = pd.Series(ratio.values, index=to_periods(ratio.index), dtype=float)</t>
-        </is>
-      </c>
+      <c r="A106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">    r = ratio.dropna().sort_index(); q = '-Q' in r.index[0]</t>
+          <t>def user_gap(credit=None, gdp=None, ratio=None, economy='User data', lamb=None, min_years=10, source='User-provided data'):</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">    lamb = lamb or (400_000 if q else 100_000)</t>
+          <t xml:space="preserve">    """Build the 3 gap rows from the user's own data, ready for chart(rows, kind='gap').</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">    tr = pd.Series(hp_one_sided(r.values, lamb), index=r.index)</t>
+          <t xml:space="preserve">    Give either `ratio` (% of GDP) or `credit` and `gdp` as pandas Series indexed by period/date.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">    tr.iloc[:min_years * (4 if q else 1)] = np.nan</t>
+          <t xml:space="preserve">    Quarterly GDP is summed over the last 4 quarters (BIS method); annual GDP with quarterly credit</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cite = f"{source}; trend and gap: own calculation, one-sided HP filter (lambda {lamb:,})"</t>
+          <t xml:space="preserve">    is matched by calendar year. lambda: 400,000 quarterly, 100,000 annual (override with lamb)."""</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">    rows = [dict(Economy=economy, **{'Indicator code': k, 'Indicator': n, 'Unit': u, 'Citation': cite, 'Source link': ''}, **s.to_dict())</t>
+          <t xml:space="preserve">    if ratio is None:</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">            for k, n, u, s in (('CREDIT_GDP', 'Credit-to-GDP ratio', 'Percent of GDP', r),</t>
+          <t xml:space="preserve">        c = pd.Series(credit.values, index=to_periods(credit.index), dtype=float).dropna()</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">                               ('CREDIT_GDP_TREND', 'Hodrick-Prescott trend', 'Percent of GDP', tr),</t>
+          <t xml:space="preserve">        g = pd.Series(gdp.values, index=to_periods(gdp.index), dtype=float).dropna()</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">                               ('CREDIT_GDP_GAP', 'Credit-to-GDP gap', 'Percentage points of GDP', r - tr))]</t>
+          <t xml:space="preserve">        qc, qg = '-Q' in c.index[0], '-Q' in g.index[0]</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">    return pd.DataFrame(rows)</t>
+          <t xml:space="preserve">        if qc and qg: g = g.sort_index().rolling(4).sum()</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr"/>
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        elif qc: g = pd.Series(g.reindex([p[:4] for p in c.index]).values, index=c.index)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr"/>
+      <c r="A118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ratio = 100 * c / g.reindex(c.index)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t># --------------------------------------------------------------------------- FSI heat map</t>
+          <t xml:space="preserve">    else:</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t># Groups and directions come from the FSI workbook: column Group, and column "More vulnerable when"</t>
+          <t xml:space="preserve">        ratio = pd.Series(ratio.values, index=to_periods(ratio.index), dtype=float)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t># ("higher" or "lower"), set from a financial-sector vulnerability perspective.</t>
+          <t xml:space="preserve">    r = ratio.dropna().sort_index(); q = '-Q' in r.index[0]</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr"/>
+      <c r="A122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    lamb = lamb or (400_000 if q else 100_000)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr"/>
+      <c r="A123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    tr = pd.Series(hp_one_sided(r.values, lamb), index=r.index)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>def percent_rank(s):</t>
+          <t xml:space="preserve">    tr.iloc[:min_years * (4 if q else 1)] = np.nan</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Excel PERCENTRANK.INC of every value within its own series: (values below) / (n - 1)."""</t>
+          <t xml:space="preserve">    cite = f"{source}; trend and gap: own calculation, one-sided HP filter (lambda {lamb:,})"</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">    s = s.dropna(); return (s.rank(method='min') - 1) / (len(s) - 1) if len(s) &gt; 1 else s * np.nan</t>
+          <t xml:space="preserve">    rows = [dict(Economy=economy, **{'Indicator code': k, 'Indicator': n, 'Unit': u, 'Citation': cite, 'Source link': ''}, **s.to_dict())</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr"/>
+      <c r="A127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            for k, n, u, s in (('CREDIT_GDP', 'Credit-to-GDP ratio', 'Percent of GDP', r),</t>
+        </is>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr"/>
+      <c r="A128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                               ('CREDIT_GDP_TREND', 'Hodrick-Prescott trend', 'Percent of GDP', tr),</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>def fsi_heatmap(country, quarters=12, min_history=8):</t>
+          <t xml:space="preserve">                               ('CREDIT_GDP_GAP', 'Credit-to-GDP gap', 'Percentage points of GDP', r - tr))]</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">    """Heat map of FSIs: colour = vulnerability percentile vs the country's own history</t>
+          <t xml:space="preserve">    return pd.DataFrame(rows)</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    (0 = least vulnerable ever, dark blue; 1 = most vulnerable ever, dark red); cells show actual values."""</t>
-        </is>
-      </c>
+      <c r="A131" t="inlineStr"/>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    rows = F[(F['Economy'].str.lower() == country.lower()) | (F['Economy code'] == country.upper())]</t>
-        </is>
-      </c>
+      <c r="A132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">    rows = rows.drop_duplicates('Indicator code').set_index('Indicator code')</t>
+          <t># --------------------------------------------------------------------------- FSI heat map</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">    per = [c for c in rows.columns if re.fullmatch(r'\d{4}-Q\d', str(c))]</t>
+          <t># Groups and directions come from the FSI workbook: column Group, and column "More vulnerable when"</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">    V = rows[per].apply(pd.to_numeric, errors='coerce')</t>
+          <t># ("higher" or "lower"), set from a financial-sector vulnerability perspective.</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    V = V[V.notna().sum(axis=1) &gt;= min_history]</t>
-        </is>
-      </c>
+      <c r="A136" t="inlineStr"/>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    rows = rows.loc[V.index]</t>
-        </is>
-      </c>
+      <c r="A137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">    R = V.apply(percent_rank, axis=1).reindex(columns=per)</t>
+          <t>def percent_rank(s):</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">    lower = (rows['More vulnerable when'] == 'lower').values; R.loc[lower] = 1 - R.loc[lower]</t>
+          <t xml:space="preserve">    """Excel PERCENTRANK.INC of every value within its own series: (values below) / (n - 1)."""</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">    first = min(V.apply(lambda r: r.first_valid_index(), axis=1).dropna())</t>
+          <t xml:space="preserve">    s = s.dropna(); return (s.rank(method='min') - 1) / (len(s) - 1) if len(s) &gt; 1 else s * np.nan</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    cols = [c for c in per if V[c].notna().any()][-quarters:]</t>
-        </is>
-      </c>
+      <c r="A141" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    V, R = V[cols], R[cols]</t>
-        </is>
-      </c>
+      <c r="A142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">    # explicit layout in inches: labels left, group names right, colour bar and source below</t>
+          <t>def fsi_heatmap(country, quarters=12, min_history=8):</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">    L = 0.3 + 0.062 * rows['Indicator'].str.len().max(); Rt = 0.4 + 0.07 * rows['Group'].str.len().max()</t>
+          <t xml:space="preserve">    """Heat map of FSIs: colour = vulnerability percentile vs the country's own history</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">    w, h, top, bot = 0.7 * len(cols), 0.42 * len(V), 0.75, 1.75</t>
+          <t xml:space="preserve">    (0 = least vulnerable ever, dark blue; 1 = most vulnerable ever, dark red); cells show actual values."""</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">    W, H = L + w + Rt, top + h + bot</t>
+          <t xml:space="preserve">    rows = F[(F['Economy'].str.lower() == country.lower()) | (F['Economy code'] == country.upper())]</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">    fig = plt.figure(figsize=(W, H)); ax = fig.add_axes([L / W, bot / H, w / W, h / H])</t>
+          <t xml:space="preserve">    rows = rows.drop_duplicates('Indicator code').set_index('Indicator code')</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">    im = ax.imshow(R.values.astype(float), cmap='RdBu_r', vmin=0, vmax=1, aspect='auto')</t>
+          <t xml:space="preserve">    per = [c for c in rows.columns if re.fullmatch(r'\d{4}-Q\d', str(c))]</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">    for i in range(len(V)):</t>
+          <t xml:space="preserve">    V = rows[per].apply(pd.to_numeric, errors='coerce')</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for j in range(len(cols)):</t>
+          <t xml:space="preserve">    V = V[V.notna().sum(axis=1) &gt;= min_history]</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">            v, r = V.iat[i, j], R.iat[i, j]</t>
+          <t xml:space="preserve">    rows = rows.loc[V.index]</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if pd.notna(v):</t>
+          <t xml:space="preserve">    R = V.apply(percent_rank, axis=1).reindex(columns=per)</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">                ax.text(j, i, f'{v:.1f}', ha='center', va='center', fontsize=8,</t>
+          <t xml:space="preserve">    lower = (rows['More vulnerable when'] == 'lower').values; R.loc[lower] = 1 - R.loc[lower]</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">                        color='white' if pd.notna(r) and abs(r - 0.5) &gt; 0.3 else 'black')</t>
+          <t xml:space="preserve">    first = min(V.apply(lambda r: r.first_valid_index(), axis=1).dropna())</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax.set_yticks(range(len(V))); ax.set_yticklabels(rows['Indicator'], fontsize=8)</t>
+          <t xml:space="preserve">    cols = [c for c in per if V[c].notna().any()][-quarters:]</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax.set_xticks(range(len(cols))); ax.set_xticklabels(cols, rotation=45, ha='right', fontsize=8)</t>
+          <t xml:space="preserve">    V, R = V[cols], R[cols]</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">    groups = list(rows['Group'])</t>
+          <t xml:space="preserve">    # explicit layout in inches: labels left, group names right, colour bar and source below</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">    starts = [i for i in range(len(groups)) if i == 0 or groups[i] != groups[i - 1]]</t>
+          <t xml:space="preserve">    L = 0.3 + 0.062 * rows['Indicator'].str.len().max(); Rt = 0.4 + 0.07 * rows['Group'].str.len().max()</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">    for i in starts[1:]: ax.axhline(i - 0.5, color='black', lw=1.2)</t>
+          <t xml:space="preserve">    w, h, top, bot = 0.7 * len(cols), 0.42 * len(V), 0.75, 1.75</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax2 = ax.twinx(); ax2.set_ylim(ax.get_ylim())</t>
+          <t xml:space="preserve">    W, H = L + w + Rt, top + h + bot</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax2.set_yticks([(s + e - 1) / 2 for s, e in zip(starts, starts[1:] + [len(groups)])])</t>
+          <t xml:space="preserve">    fig = plt.figure(figsize=(W, H)); ax = fig.add_axes([L / W, bot / H, w / W, h / H])</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax2.set_yticklabels([groups[s] for s in starts], fontsize=8, weight='bold', color=BLUE)</t>
+          <t xml:space="preserve">    im = ax.imshow(R.values.astype(float), cmap='RdBu_r', vmin=0, vmax=1, aspect='auto')</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax2.tick_params(length=0); ax2.spines[:].set_visible(False)</t>
+          <t xml:space="preserve">    for i in range(len(V)):</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cax = fig.add_axes([L / W, 0.55 / H, min(w, 5) / W, 0.13 / H])</t>
+          <t xml:space="preserve">        for j in range(len(cols)):</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cb = fig.colorbar(im, cax=cax, orientation='horizontal'); cb.set_ticks([0, 0.5, 1])</t>
+          <t xml:space="preserve">            v, r = V.iat[i, j], R.iat[i, j]</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cb.set_ticklabels(['Less vulnerable', 'Median', 'More vulnerable']); cb.ax.tick_params(labelsize=8)</t>
+          <t xml:space="preserve">            if pd.notna(v):</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ax.set_title(f"{rows['Economy'].dropna().iloc[0]}: financial soundness heat map\n"</t>
+          <t xml:space="preserve">                ax.text(j, i, f'{v:.1f}', ha='center', va='center', fontsize=8,</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 "colour = percent rank vs own history (dark red = most vulnerable, dark blue = least)",</t>
+          <t xml:space="preserve">                        color='white' if pd.notna(r) and abs(r - 0.5) &gt; 0.3 else 'black')</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 loc='left', weight='bold', color=BLUE, fontsize=10)</t>
+          <t xml:space="preserve">    ax.set_yticks(range(len(V))); ax.set_yticklabels(rows['Indicator'], fontsize=8)</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t xml:space="preserve">    note = f"Each indicator is ranked against all its own quarters since {first} (Excel PERCENTRANK.INC)."</t>
+          <t xml:space="preserve">    ax.set_xticks(range(len(cols))); ax.set_xticklabels(cols, rotation=45, ha='right', fontsize=8)</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t xml:space="preserve">    fig.text(0.01, 0.06 / H, textwrap.fill(f"Source: {rows['Citation'].dropna().iloc[0]}. {note}", int(W * 14)),</t>
+          <t xml:space="preserve">    groups = list(rows['Group'])</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t xml:space="preserve">             fontsize=8, color='dimgray'); plt.show()</t>
+          <t xml:space="preserve">    starts = [i for i in range(len(groups)) if i == 0 or groups[i] != groups[i - 1]]</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t xml:space="preserve">    return pd.DataFrame({'Group': rows['Group'].values, 'Indicator': rows['Indicator'].values,</t>
+          <t xml:space="preserve">    for i in starts[1:]: ax.axhline(i - 0.5, color='black', lw=1.2)</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t xml:space="preserve">                         'Latest value': V.ffill(axis=1).iloc[:, -1].round(2).values,</t>
+          <t xml:space="preserve">    ax2 = ax.twinx(); ax2.set_ylim(ax.get_ylim())</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ax2.set_yticks([(s + e - 1) / 2 for s, e in zip(starts, starts[1:] + [len(groups)])])</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ax2.set_yticklabels([groups[s] for s in starts], fontsize=8, weight='bold', color=BLUE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ax2.tick_params(length=0); ax2.spines[:].set_visible(False)</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    cax = fig.add_axes([L / W, 0.55 / H, min(w, 5) / W, 0.13 / H])</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    cb = fig.colorbar(im, cax=cax, orientation='horizontal'); cb.set_ticks([0, 0.5, 1])</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    cb.set_ticklabels(['Less vulnerable', 'Median', 'More vulnerable']); cb.ax.tick_params(labelsize=8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ax.set_title(f"{rows['Economy'].dropna().iloc[0]}: financial soundness heat map\n"</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 "colour = percent rank vs own history (dark red = most vulnerable, dark blue = least)",</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 loc='left', weight='bold', color=BLUE, fontsize=10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    note = f"Each indicator is ranked against all its own quarters since {first} (Excel PERCENTRANK.INC)."</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    fig.text(0.01, 0.06 / H, textwrap.fill(f"Source: {rows['Citation'].dropna().iloc[0]}. {note}", int(W * 14)),</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             fontsize=8, color='dimgray'); plt.show()</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    return pd.DataFrame({'Group': rows['Group'].values, 'Indicator': rows['Indicator'].values,</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         'Latest value': V.ffill(axis=1).iloc[:, -1].round(2).values,</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
         <is>
           <t xml:space="preserve">                         'Vulnerability percentile': R.ffill(axis=1).iloc[:, -1].round(2).values})</t>
         </is>

</xml_diff>